<commit_message>
Adjust item 8 handling and regenerate outputs
Commented-out code in Fit_3PL_Fix_3EM_MT_S1.R that removed rpa_008/Item rpa_008 so the item is no longer automatically excluded. Updated gera_relatorio_3EM_MT.py to reflect that item 8 from Simulado I was retained in the TRI with a technical caveat: changed lead text, the item table entry, risk paragraph, and recommendations. Also improved parameter-summary formatting (compute counts once and handle singular/plural). Regenerated binary report artifacts (docx, xlsx, pdf) in Relatorios and ResultadosTRI/Simulado_I to reflect these changes.
</commit_message>
<xml_diff>
--- a/Piaui/2026/ResultadosTRI_3EM_MT/Simulado_I/DistriAlunosClasseMT3serie_S1.xlsx
+++ b/Piaui/2026/ResultadosTRI_3EM_MT/Simulado_I/DistriAlunosClasseMT3serie_S1.xlsx
@@ -473,10 +473,10 @@
         <v>9</v>
       </c>
       <c r="B8" t="n">
-        <v>449</v>
+        <v>1084</v>
       </c>
       <c r="C8" t="n">
-        <v>1.58</v>
+        <v>3.815</v>
       </c>
     </row>
     <row r="9">
@@ -484,10 +484,10 @@
         <v>10</v>
       </c>
       <c r="B9" t="n">
-        <v>4398</v>
+        <v>4308</v>
       </c>
       <c r="C9" t="n">
-        <v>15.477</v>
+        <v>15.16</v>
       </c>
     </row>
     <row r="10">
@@ -495,10 +495,10 @@
         <v>11</v>
       </c>
       <c r="B10" t="n">
-        <v>5028</v>
+        <v>5671</v>
       </c>
       <c r="C10" t="n">
-        <v>17.694</v>
+        <v>19.957</v>
       </c>
     </row>
     <row r="11">
@@ -506,10 +506,10 @@
         <v>12</v>
       </c>
       <c r="B11" t="n">
-        <v>4636</v>
+        <v>4806</v>
       </c>
       <c r="C11" t="n">
-        <v>16.315</v>
+        <v>16.913</v>
       </c>
     </row>
     <row r="12">
@@ -517,10 +517,10 @@
         <v>13</v>
       </c>
       <c r="B12" t="n">
-        <v>3570</v>
+        <v>3371</v>
       </c>
       <c r="C12" t="n">
-        <v>12.563</v>
+        <v>11.863</v>
       </c>
     </row>
     <row r="13">
@@ -528,10 +528,10 @@
         <v>14</v>
       </c>
       <c r="B13" t="n">
-        <v>2349</v>
+        <v>2199</v>
       </c>
       <c r="C13" t="n">
-        <v>8.266</v>
+        <v>7.739</v>
       </c>
     </row>
     <row r="14">
@@ -539,10 +539,10 @@
         <v>15</v>
       </c>
       <c r="B14" t="n">
-        <v>1811</v>
+        <v>1957</v>
       </c>
       <c r="C14" t="n">
-        <v>6.373</v>
+        <v>6.887</v>
       </c>
     </row>
     <row r="15">
@@ -550,10 +550,10 @@
         <v>16</v>
       </c>
       <c r="B15" t="n">
-        <v>6175</v>
+        <v>5020</v>
       </c>
       <c r="C15" t="n">
-        <v>21.731</v>
+        <v>17.666</v>
       </c>
     </row>
   </sheetData>

</xml_diff>